<commit_message>
Add 11 independently verified Nankai profiles (1026 records)
</commit_message>
<xml_diff>
--- a/site/exports/nku-history.xlsx
+++ b/site/exports/nku-history.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'总览'!$A$1:$K$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'经历'!$A$1:$S$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'导师'!$A$1:$L$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'论文'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'来源'!$A$1:$G$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -452,7 +452,7 @@
     <col width="65" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="65" customWidth="1" min="6" max="6"/>
-    <col width="37.8" customWidth="1" min="7" max="7"/>
+    <col width="65" customWidth="1" min="7" max="7"/>
     <col width="26.6" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
@@ -569,10 +569,118 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>历史学院</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>原目录列教授、博士生导师、讲席教授；博士生导师为本人指导资格，不推本人导师。目录与原开放任期不是实时人事核验。；硕士两个官网分别记1990-01学习终点和1989毕业，博士分别记1996-09至1999-07学习与1996毕业；一个阶段仅一个学位，冲突规范日期留空。；中国农科院起年1984-08与1986不一致，不选一方；历史系/历史学院副院长名称差异保留，晋升起点不由入职日期猜。；海德堡2004/2005可能不同访问，事件对应未知；堪萨斯原2012/04-2005/05倒置不纠正。；官网两条署名王乾只作身份未解书目提及，不计王利华作品，不认别名、不另建或合并人物；本人已接受作品0条不等没有作品。</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；部分必要职业资料，非完整履历；公开教学事实（非本人求学学历；教学／课程开设时间不是入学、授位或任职起点；不计入教育、任职、论文、导师统计及师承图）：本科生课程：中国古代后期史、中国古代经济史、中国生态环境变迁史（中国生态环境史）、隋唐五代史、中国文明史、生态文明等。；主讲；教学／课程开设时间：时间未披露；本科生课程；页面合述曾经主讲和目前主讲，不能逐门指定当前状态。；来源ID：nku-wanglihua-history-profile；https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm | 研究生课程：隋唐五代史专题研究、隋唐五代史料、古代经济史专题、古代经济文献选读。；主讲；教学／课程开设时间：时间未披露；研究生课程；页面合述曾经主讲和目前主讲，不能逐门指定当前状态。；来源ID：nku-wanglihua-history-profile；https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm | 中国环境史概论、中国环境史资料整理与研究、环境史导论等。；主讲；教学／课程开设时间：时间未披露；未单独标明层次；页面合述曾经主讲和目前主讲，不能逐门指定当前状态。；来源ID：nku-wanglihua-history-profile；https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>江沛</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>校区未标注</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>历史学院</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>原南开大学历史学院教授身份，教授起任日期未知；1989起任教不回溯为教授职称起任。；原1982至1989合并学习区间先后获历史学学士、硕士，不拆分学段边界或授位日期；2000年6月博士授位明确保留。；2000年6月至2003年3月南京大学历史学博士后原明确完成，非学位且不重复任职。；本人导师未披露；两选录主要著作作者表未给，不认独著或自补作者，原出版月份与第3卷保留。</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>分批核实资料，不是完整名录；人物整体核验日期未单独记录</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>公开个人页（访问与内容时效见来源记录）</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:K4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -584,11 +692,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:S27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="30.8" customWidth="1" min="2" max="2"/>
     <col width="33.59999999999999" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
@@ -1159,8 +1267,1098 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>历史学学士</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>北京大学</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>1980-09</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>1984-07</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>1980/09-1984/07  北京大学学习，获历史学学士学位。 原文明确获学位，授位true；学习/毕业时间不独立等同授位日，法律授位实体未核。</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>农学硕士</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>南京农业大学</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1986-09</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>1986/09-1990/01  南京农业大学学习，获农学硕士学位。 原文明确获学位，授位true；学习/毕业时间不独立等同授位日，法律授位实体未核。 两官网硕士毕业时间冲突，end不取任一版本；非两个硕士学位。 两官网另列1989年毕业与1990年1月学习终点，未择一改写。</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>历史学博士</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>1996/09-1999/07  南开大学学习，获历史学博士学位。 原文明确获学位，授位true；学习/毕业时间不独立等同授位日，法律授位实体未核。 两官网博士学习及毕业时间冲突，规范start/end均留空；非两个博士学位。 两官网另列1996年毕业与1996-09至1999-07学习区间，未择一改写。</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>visiting_research</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>访问研究</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>韩国成均馆大学</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2002-09</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>2003-08</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>2002/09-2003/08，韩国成均馆大学访问研究。 非学位职业访问，不据此推授位或本人导师。</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr"/>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>academic_lecture_visit</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>讲学</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>德国海德堡大学</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>2005/05-2005/07，德国海德堡大学讲学。 两官网德国讲学分别记2005和2004；可能是不同访问，未确认同一事件，故合为访问记录组且规范日期空，不断言某版本错误或只有一次访问。 另一官网原2004年短期讲学并任客座教授；不强称同一次访问。</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr"/>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>visiting_research</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>访问研究</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>美国堪萨斯大学</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>2012/04-2005/05，美国堪萨斯大学访问研究。 原文2012/04-2005/05次序倒置。保留原摘录，不猜测2005应为2012或2013，规范start/end空。</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr"/>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>研究实习员、助理研究员、副研究员（先后）</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>中国农业科学院中国农业遗产研究室</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>1999-10</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>1984/08-1999/10，中国农业科学院中国农业遗产研究室研究实习员、助理研究员、副研究员，1995年获中国农业科学院跨世纪学科带头人提名，列入重点培养对象。 起年1984/1986冲突不裁决，职称晋升年份未知；末年1999与1999-10精度不同，不强称冲突。 原另一官网1986—1999起年与1984-08不一致；1995提名/1996相关记载并存，不校正；职称先后并列，不拆晋升日期。</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr"/>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>副教授</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>南开大学历史系</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>1999-11</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2003-12</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1999/11-2003/12，南开大学历史系副教授。 </t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr"/>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>教授</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>南开大学历史系</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2003-12</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>2003/12-，南开大学历史系教授，次年起担任博士生导师。  原次年起担任博士生导师，即2004年指导资格，不另作任职或本人导师。 原开放任期不认证实时现任。</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr"/>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>副院长（主管教学工作）</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2004-01</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2015-05</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>2004/01-2015/05，南开大学历史系副院长（主管教学工作）。 同页历史系/历史学院名称不一致，规范机构仅南开大学；不凭副院长称谓改写来源。 同页另称历史学院副院长，原历史系/学院两名称并列，机构不自行纠正。</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr"/>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>副院长</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>南开大学生态文明研究院</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2015-11</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>2015/11-，南开大学生态文明研究院副院长。  原开放任期不认证实时现任。</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>杰出教授岗位</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2016-01</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2016/01-2026/08，南开大学杰出教授岗位。 </t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr"/>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>讲席教授岗位</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>2026/08-，南开大学讲席教授岗位。  原开放任期不认证实时现任。</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr"/>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>江沛</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>历史学学士</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>南开大学历史系</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>原1982至1989合并学习区间，先后获历史学学士、硕士学位；本条为历史学学士，个别学段起止与授位年月未披露。</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr"/>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>江沛</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>历史学硕士</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>南开大学历史系</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>原1982至1989合并学习区间，先后获历史学学士、硕士学位；本条为历史学硕士，个别学段起止与授位年月未披露。</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr"/>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>江沛</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>degree</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>历史学博士</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>2000-06</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>原2000年6月获南开大学历史学博士学位，保留明确授位月份。</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr"/>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>江沛</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>postdoctoral_research</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>非学位</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>南京大学历史学博士后流动站</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2000-06</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>2003-03</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>原2000年6月至2003年3月完成南京大学历史学博士后研究工作，非学位，不再重复计任职。</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr"/>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>江沛</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>employment</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>任教</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>南开大学历史学系、历史学院</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>原1989年起至今在南开大学历史学系、历史学院任教；教授身份另列，教授起任日未知，不把任教起点当教授起任。原至今不认证实时现任。</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr"/>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:S9"/>
+  <autoFilter ref="A1:S27"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId2"/>
@@ -1170,6 +2368,24 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1272,7 +2488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1455,13 +2671,121 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>江沛</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>战国策派思潮研究</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2001</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>官网书目，未核出版者元数据或全文；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>个人主要著作或成果列目，完整作者表和具体著编贡献未披露，不推独著；天津人民出版社，2001年8月。</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>江沛</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>国民党结构史论</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>2013</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>book</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>官网书目，未核出版者元数据或全文；official_publication_list_only</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>个人主要著作或成果列目，完整作者表和具体著编贡献未披露，不推独著；中华书局，2013年1月。原第3卷。</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L3"/>
+  <autoFilter ref="A1:L5"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1473,7 +2797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1633,12 +2957,164 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>nku-wanglihua-history-profile</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c16087a201695/page.htm</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>retained_professional_excerpts_checked</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>nku-wanglihua-ccsh-profile</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>https://ccsh.nankai.edu.cn/2020/1230/c22202a332233/page.htm</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>retained_professional_excerpts_checked</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>王利华</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>nku-history-directory</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/16054/list.htm</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>original_person_directory_metadata_only</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>江沛</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>nku-1-387</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://history.nankai.edu.cn/2019/0910/c34459a560699/page.htm</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>retained_professional_excerpts_checked</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>nku</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>南开大学</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:G8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>